<commit_message>
audit(avis-dataforseo-api-seo): enrich 2026-06-09 snapshot with thruuu serp & AI comparison data
</commit_message>
<xml_diff>
--- a/content/audits/avis-dataforseo-api-seo/2026-06-09/avis-dataforseo-volumes-seo.xlsx
+++ b/content/audits/avis-dataforseo-api-seo/2026-06-09/avis-dataforseo-volumes-seo.xlsx
@@ -10,6 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cluster cible" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champ sémantique" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SERP Comparative" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SERP Thruuu" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topics Thruuu" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FAQ Thruuu" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1184,4 +1187,3651 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Organic Position</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Hostname</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Word Count</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Image Count</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Schema Type</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Has SERP FAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>reddit.com</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Reddit - The heart of the internet</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/SEO/comments/1npkyh8/dataforseo_how_good_is_it/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>132</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>dataforseo.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Powerful API Stack For Data-Driven SEO Tools – DataForSEO</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://dataforseo.com/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>941</v>
+      </c>
+      <c r="G3" t="n">
+        <v>73</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Place,LegalService,Organization,WebSite,ImageObject,WebPage,Person,Article</t>
+        </is>
+      </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>trustpilot.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>DataForSEO Reviews | Read Customer Service Reviews of dataforseo.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://www.trustpilot.com/review/dataforseo.com</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1852</v>
+      </c>
+      <c r="G4" t="n">
+        <v>47</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Organization,ImageObject (2),WebSite,WebPage,BreadcrumbList,LocalBusiness,Review (20),Dataset</t>
+        </is>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>comparatif-logiciels.fr</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>DataForSEO: présentation, avis clients &amp; tarifs</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://www.comparatif-logiciels.fr/avis-dataforseo/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>259</v>
+      </c>
+      <c r="G5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Organization,WebSite,ImageObject,WebPage,Person,SoftwareApplication,BreadcrumbList</t>
+        </is>
+      </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>reddit.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Reddit - The heart of the internet</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/TechSEO/comments/1s4tbt6/what_an_terrible_user_experience_that_dataforseo/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>277</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>dataforseo.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Integrations – DataForSEO</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://dataforseo.com/integrations</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>491</v>
+      </c>
+      <c r="G7" t="n">
+        <v>63</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Place,LegalService,Organization,WebSite,ImageObject,BreadcrumbList,WebPage,Person,Article</t>
+        </is>
+      </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B8" t="n">
+        <v>8</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>nextgrowth.ai</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DataForSEO Review 2026: Honest Verdict After 12 Weeks</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://nextgrowth.ai/dataforseo-review/</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>3782</v>
+      </c>
+      <c r="G8" t="n">
+        <v>17</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Organization,WebSite,ImageObject,BreadcrumbList,WebPage,Person (2),BlogPosting,Review,FAQPage</t>
+        </is>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B9" t="n">
+        <v>9</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>logiciels.pro</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>DataForSEO: avis, prix, fonctionnalités &amp; alternatives</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.logiciels.pro/logiciel-saas/dataforseo/</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>556</v>
+      </c>
+      <c r="G9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Organization,WebSite,ImageObject,WebPage,Person,SoftwareApplication,BreadcrumbList</t>
+        </is>
+      </c>
+      <c r="I9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" t="n">
+        <v>10</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>dataforseo.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Business Data API by DataForSEO | Company Information and Reviews Data API</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://dataforseo.com/apis/business-data-api</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>658</v>
+      </c>
+      <c r="G10" t="n">
+        <v>55</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Place,LegalService,Organization,WebSite,ImageObject,BreadcrumbList,WebPage,SoftwareApplication</t>
+        </is>
+      </c>
+      <c r="I10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>11</v>
+      </c>
+      <c r="B11" t="n">
+        <v>11</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>marketing-tools.tech</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Client Challenge</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://www.marketing-tools.tech/dataforseo/</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>12</v>
+      </c>
+      <c r="B12" t="n">
+        <v>12</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>dataforseo.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>DataForSEO vs Competitors – DataForSEO</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://dataforseo.com/blog/category/competitor-comparisons</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>211</v>
+      </c>
+      <c r="G12" t="n">
+        <v>11</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Place,LegalService,WebSite,BreadcrumbList,CollectionPage</t>
+        </is>
+      </c>
+      <c r="I12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>13</v>
+      </c>
+      <c r="B13" t="n">
+        <v>13</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>g2.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>DataForSEO Pros and Cons | User Likes &amp; Dislikes</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://www.g2.com/products/dataforseo/reviews</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>14</v>
+      </c>
+      <c r="B14" t="n">
+        <v>14</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>hellip.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>DataForSEO. À propos, connecteurs, intégrations</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://hellip.com/fr/product/dataforseo.html</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>725</v>
+      </c>
+      <c r="G14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>15</v>
+      </c>
+      <c r="B15" t="n">
+        <v>15</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>dataforseo.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Getting Reviews &amp; Ratings Data at a Low Cost with API from DataForSEO – DataForSEO</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://dataforseo.com/blog/scraping-reviews-with-dataforseo-api</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>2777</v>
+      </c>
+      <c r="G15" t="n">
+        <v>14</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Place,LegalService,Organization,WebSite,ImageObject,BreadcrumbList,WebPage,Person,BlogPosting</t>
+        </is>
+      </c>
+      <c r="I15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>16</v>
+      </c>
+      <c r="B16" t="n">
+        <v>16</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>thatmarketingbuddy.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>DataForSEO Review 2026: API-First Data Platform for SEO Builders | TMB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://thatmarketingbuddy.com/software/dataforseo</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1835</v>
+      </c>
+      <c r="G16" t="n">
+        <v>15</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Organization,WebSite,Person,BreadcrumbList,SoftwareApplication,Product,FAQPage</t>
+        </is>
+      </c>
+      <c r="I16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>17</v>
+      </c>
+      <c r="B17" t="n">
+        <v>17</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>trustradius.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>DataForSEO Reviews &amp; Ratings 2026</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://www.trustradius.com/products/dataforseo/reviews</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>18</v>
+      </c>
+      <c r="B18" t="n">
+        <v>18</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>dataforseo.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Reviews API – DataForSEO</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://dataforseo.com/apis/reviews-api</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>909</v>
+      </c>
+      <c r="G18" t="n">
+        <v>53</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Place,LegalService,Organization,WebSite,ImageObject,BreadcrumbList,WebPage,Person,Article</t>
+        </is>
+      </c>
+      <c r="I18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>19</v>
+      </c>
+      <c r="B19" t="n">
+        <v>19</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>comparatif-logiciels.fr</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>DataForSEO: présentation, avis clients &amp; tarifs</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://www.comparatif-logiciels.fr/logiciel/avis-dataforseo/</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>259</v>
+      </c>
+      <c r="G19" t="n">
+        <v>6</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Organization,WebSite,ImageObject,WebPage,Person,SoftwareApplication,BreadcrumbList</t>
+        </is>
+      </c>
+      <c r="I19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>20</v>
+      </c>
+      <c r="B20" t="n">
+        <v>20</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>elitecontentmarketer.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>DataForSEO Review – Elite Content Marketer</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://www.elitecontentmarketer.com/stack/dataforseo/</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>103</v>
+      </c>
+      <c r="G20" t="n">
+        <v>6</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Organization,WebSite,BreadcrumbList,SoftwareApplication</t>
+        </is>
+      </c>
+      <c r="I20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D160"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Found in Pages</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Total Frequency</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Relevancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>reddit</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3.194444444444445</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>of</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3" t="n">
+        <v>88</v>
+      </c>
+      <c r="D3" t="n">
+        <v>20.25</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>7</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.111111111111111</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>the</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C5" t="n">
+        <v>175</v>
+      </c>
+      <c r="D5" t="n">
+        <v>31.92314814814815</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>privacy</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>18</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.592592592592593</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>of reddit</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.555555555555556</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>best of</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="n">
+        <v>6</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1.555555555555556</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>best of reddit</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.333333333333333</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>of reddit in</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1.555555555555556</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>and</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" t="n">
+        <v>183</v>
+      </c>
+      <c r="D12" t="n">
+        <v>24.23148148148148</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" t="n">
+        <v>138</v>
+      </c>
+      <c r="D13" t="n">
+        <v>20.10515873015873</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>dataforseo</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>7</v>
+      </c>
+      <c r="C14" t="n">
+        <v>259</v>
+      </c>
+      <c r="D14" t="n">
+        <v>38.5891975308642</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>our</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="n">
+        <v>52</v>
+      </c>
+      <c r="D15" t="n">
+        <v>7.166666666666667</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>api</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>7</v>
+      </c>
+      <c r="C16" t="n">
+        <v>115</v>
+      </c>
+      <c r="D16" t="n">
+        <v>19.29907407407408</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>seo</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" t="n">
+        <v>78</v>
+      </c>
+      <c r="D17" t="n">
+        <v>11.2494708994709</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>with</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" t="n">
+        <v>75</v>
+      </c>
+      <c r="D18" t="n">
+        <v>9.677248677248677</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>is</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" t="n">
+        <v>97</v>
+      </c>
+      <c r="D19" t="n">
+        <v>11.84920634920635</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>your</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" t="n">
+        <v>60</v>
+      </c>
+      <c r="D20" t="n">
+        <v>7.439814814814814</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" t="n">
+        <v>86</v>
+      </c>
+      <c r="D21" t="n">
+        <v>9.932539682539684</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>you</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C22" t="n">
+        <v>82</v>
+      </c>
+      <c r="D22" t="n">
+        <v>10.38624338624339</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>tool</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" t="n">
+        <v>47</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4.385714285714285</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>for</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>5</v>
+      </c>
+      <c r="C24" t="n">
+        <v>114</v>
+      </c>
+      <c r="D24" t="n">
+        <v>12.82671957671958</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>we</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" t="n">
+        <v>35</v>
+      </c>
+      <c r="D25" t="n">
+        <v>4.166666666666667</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>dataforseo api</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" t="n">
+        <v>26</v>
+      </c>
+      <c r="D26" t="n">
+        <v>4.304761904761905</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>solution</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" t="n">
+        <v>19</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1.89047619047619</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>can</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>5</v>
+      </c>
+      <c r="C28" t="n">
+        <v>31</v>
+      </c>
+      <c r="D28" t="n">
+        <v>5.0760582010582</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>with dataforseo</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" t="n">
+        <v>21</v>
+      </c>
+      <c r="D29" t="n">
+        <v>4.225396825396825</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" t="n">
+        <v>15</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1.333333333333333</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>build</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" t="n">
+        <v>17</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1.40952380952381</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>by</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C32" t="n">
+        <v>21</v>
+      </c>
+      <c r="D32" t="n">
+        <v>2.688888888888889</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>backlink</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>4</v>
+      </c>
+      <c r="C33" t="n">
+        <v>20</v>
+      </c>
+      <c r="D33" t="n">
+        <v>2.344444444444445</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" t="n">
+        <v>9</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>most</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>4</v>
+      </c>
+      <c r="C35" t="n">
+        <v>21</v>
+      </c>
+      <c r="D35" t="n">
+        <v>2.468253968253968</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>are</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" t="n">
+        <v>25</v>
+      </c>
+      <c r="D36" t="n">
+        <v>2.486111111111111</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" t="n">
+        <v>43</v>
+      </c>
+      <c r="D37" t="n">
+        <v>4.362962962962963</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>help</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>4</v>
+      </c>
+      <c r="C38" t="n">
+        <v>19</v>
+      </c>
+      <c r="D38" t="n">
+        <v>2.285185185185185</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>4</v>
+      </c>
+      <c r="C39" t="n">
+        <v>34</v>
+      </c>
+      <c r="D39" t="n">
+        <v>3.037037037037037</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" t="n">
+        <v>31</v>
+      </c>
+      <c r="D40" t="n">
+        <v>3.462962962962963</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" t="n">
+        <v>13</v>
+      </c>
+      <c r="D41" t="n">
+        <v>1.148148148148148</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>4</v>
+      </c>
+      <c r="C42" t="n">
+        <v>17</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1.719753086419753</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>the most</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>3</v>
+      </c>
+      <c r="C43" t="n">
+        <v>11</v>
+      </c>
+      <c r="D43" t="n">
+        <v>2.202380952380952</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C44" t="n">
+        <v>40</v>
+      </c>
+      <c r="D44" t="n">
+        <v>2.847222222222222</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>how</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>4</v>
+      </c>
+      <c r="C45" t="n">
+        <v>29</v>
+      </c>
+      <c r="D45" t="n">
+        <v>2.603703703703704</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>guide</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>3</v>
+      </c>
+      <c r="C46" t="n">
+        <v>21</v>
+      </c>
+      <c r="D46" t="n">
+        <v>1.341666666666667</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>3</v>
+      </c>
+      <c r="C47" t="n">
+        <v>10</v>
+      </c>
+      <c r="D47" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>keyword research</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>3</v>
+      </c>
+      <c r="C48" t="n">
+        <v>11</v>
+      </c>
+      <c r="D48" t="n">
+        <v>1.85</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" t="n">
+        <v>8</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0.5333333333333333</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>reputation</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" t="n">
+        <v>8</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0.5333333333333333</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>reputation management</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="n">
+        <v>8</v>
+      </c>
+      <c r="D51" t="n">
+        <v>1.066666666666667</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>3</v>
+      </c>
+      <c r="C52" t="n">
+        <v>16</v>
+      </c>
+      <c r="D52" t="n">
+        <v>1.133333333333333</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>out</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="n">
+        <v>7</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>building</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" t="n">
+        <v>7</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0.5277777777777778</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="n">
+        <v>10</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0.6111111111111112</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>that</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" t="n">
+        <v>30</v>
+      </c>
+      <c r="D56" t="n">
+        <v>2.444444444444445</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>access</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" t="n">
+        <v>10</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0.6111111111111112</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>case</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>2</v>
+      </c>
+      <c r="C58" t="n">
+        <v>7</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0.5277777777777778</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>find</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>2</v>
+      </c>
+      <c r="C59" t="n">
+        <v>7</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0.5111111111111111</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>use case</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>2</v>
+      </c>
+      <c r="C60" t="n">
+        <v>7</v>
+      </c>
+      <c r="D60" t="n">
+        <v>1.055555555555556</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>usage</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>2</v>
+      </c>
+      <c r="C61" t="n">
+        <v>11</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0.5555555555555556</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>3</v>
+      </c>
+      <c r="C62" t="n">
+        <v>17</v>
+      </c>
+      <c r="D62" t="n">
+        <v>1.361111111111111</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>you can</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C63" t="n">
+        <v>12</v>
+      </c>
+      <c r="D63" t="n">
+        <v>2.222222222222222</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>how to</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>2</v>
+      </c>
+      <c r="C64" t="n">
+        <v>6</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>guide to</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>2</v>
+      </c>
+      <c r="C65" t="n">
+        <v>6</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>engine</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" t="n">
+        <v>6</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0.4074074074074074</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>search engine</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>2</v>
+      </c>
+      <c r="C67" t="n">
+        <v>6</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0.8148148148148148</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>tracking</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>3</v>
+      </c>
+      <c r="C68" t="n">
+        <v>11</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0.8083333333333332</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>rank tracking</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>3</v>
+      </c>
+      <c r="C69" t="n">
+        <v>11</v>
+      </c>
+      <c r="D69" t="n">
+        <v>1.616666666666666</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>2</v>
+      </c>
+      <c r="C70" t="n">
+        <v>20</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0.7111111111111111</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>to build</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>2</v>
+      </c>
+      <c r="C71" t="n">
+        <v>7</v>
+      </c>
+      <c r="D71" t="n">
+        <v>0.8444444444444444</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>of the</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>2</v>
+      </c>
+      <c r="C72" t="n">
+        <v>9</v>
+      </c>
+      <c r="D72" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" t="n">
+        <v>6</v>
+      </c>
+      <c r="D73" t="n">
+        <v>0.5555555555555556</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>committed</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>2</v>
+      </c>
+      <c r="C74" t="n">
+        <v>6</v>
+      </c>
+      <c r="D74" t="n">
+        <v>0.5555555555555556</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>2</v>
+      </c>
+      <c r="C75" t="n">
+        <v>7</v>
+      </c>
+      <c r="D75" t="n">
+        <v>0.4444444444444444</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>is the</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>2</v>
+      </c>
+      <c r="C76" t="n">
+        <v>10</v>
+      </c>
+      <c r="D76" t="n">
+        <v>1.055555555555556</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>they</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>3</v>
+      </c>
+      <c r="C77" t="n">
+        <v>22</v>
+      </c>
+      <c r="D77" t="n">
+        <v>2.402777777777778</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>3</v>
+      </c>
+      <c r="C78" t="n">
+        <v>18</v>
+      </c>
+      <c r="D78" t="n">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>reliable</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>2</v>
+      </c>
+      <c r="C79" t="n">
+        <v>9</v>
+      </c>
+      <c r="D79" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>what</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>3</v>
+      </c>
+      <c r="C80" t="n">
+        <v>26</v>
+      </c>
+      <c r="D80" t="n">
+        <v>1.736111111111111</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>get</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>4</v>
+      </c>
+      <c r="C81" t="n">
+        <v>16</v>
+      </c>
+      <c r="D81" t="n">
+        <v>2.003703703703704</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>with dataforseo api</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>2</v>
+      </c>
+      <c r="C82" t="n">
+        <v>6</v>
+      </c>
+      <c r="D82" t="n">
+        <v>0.9333333333333331</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>own keyword research</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>2</v>
+      </c>
+      <c r="C83" t="n">
+        <v>4</v>
+      </c>
+      <c r="D83" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>your own keyword</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>2</v>
+      </c>
+      <c r="C84" t="n">
+        <v>4</v>
+      </c>
+      <c r="D84" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>reputation management tool</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>2</v>
+      </c>
+      <c r="C85" t="n">
+        <v>4</v>
+      </c>
+      <c r="D85" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>dataforseo backlinks api</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>2</v>
+      </c>
+      <c r="C86" t="n">
+        <v>4</v>
+      </c>
+      <c r="D86" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>with dataforseo backlinks</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>2</v>
+      </c>
+      <c r="C87" t="n">
+        <v>4</v>
+      </c>
+      <c r="D87" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>find out how</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>2</v>
+      </c>
+      <c r="C88" t="n">
+        <v>4</v>
+      </c>
+      <c r="D88" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>learn how to</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>2</v>
+      </c>
+      <c r="C89" t="n">
+        <v>4</v>
+      </c>
+      <c r="D89" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>tool with dataforseo</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>2</v>
+      </c>
+      <c r="C90" t="n">
+        <v>4</v>
+      </c>
+      <c r="D90" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>tracking tool with</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>2</v>
+      </c>
+      <c r="C91" t="n">
+        <v>4</v>
+      </c>
+      <c r="D91" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>rank tracking tool</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>2</v>
+      </c>
+      <c r="C92" t="n">
+        <v>4</v>
+      </c>
+      <c r="D92" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>our guide to</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>2</v>
+      </c>
+      <c r="C93" t="n">
+        <v>4</v>
+      </c>
+      <c r="D93" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>3</v>
+      </c>
+      <c r="C94" t="n">
+        <v>55</v>
+      </c>
+      <c r="D94" t="n">
+        <v>3.736111111111111</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>2</v>
+      </c>
+      <c r="C95" t="n">
+        <v>35</v>
+      </c>
+      <c r="D95" t="n">
+        <v>1.898148148148148</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>com</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>2</v>
+      </c>
+      <c r="C96" t="n">
+        <v>27</v>
+      </c>
+      <c r="D96" t="n">
+        <v>1.444444444444444</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>this</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>2</v>
+      </c>
+      <c r="C97" t="n">
+        <v>28</v>
+      </c>
+      <c r="D97" t="n">
+        <v>1.472222222222222</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>not</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>2</v>
+      </c>
+      <c r="C98" t="n">
+        <v>29</v>
+      </c>
+      <c r="D98" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>more</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>4</v>
+      </c>
+      <c r="C99" t="n">
+        <v>28</v>
+      </c>
+      <c r="D99" t="n">
+        <v>2.74973544973545</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>like</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>2</v>
+      </c>
+      <c r="C100" t="n">
+        <v>17</v>
+      </c>
+      <c r="D100" t="n">
+        <v>0.9351851851851851</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>have</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>2</v>
+      </c>
+      <c r="C101" t="n">
+        <v>15</v>
+      </c>
+      <c r="D101" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>or</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>2</v>
+      </c>
+      <c r="C102" t="n">
+        <v>25</v>
+      </c>
+      <c r="D102" t="n">
+        <v>1.064814814814815</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>if</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>2</v>
+      </c>
+      <c r="C103" t="n">
+        <v>20</v>
+      </c>
+      <c r="D103" t="n">
+        <v>0.8796296296296295</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>re</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>2</v>
+      </c>
+      <c r="C104" t="n">
+        <v>12</v>
+      </c>
+      <c r="D104" t="n">
+        <v>0.6111111111111112</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>serp</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>2</v>
+      </c>
+      <c r="C105" t="n">
+        <v>25</v>
+      </c>
+      <c r="D105" t="n">
+        <v>0.9722222222222222</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>if you</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>2</v>
+      </c>
+      <c r="C106" t="n">
+        <v>11</v>
+      </c>
+      <c r="D106" t="n">
+        <v>1.166666666666667</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>do</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>2</v>
+      </c>
+      <c r="C107" t="n">
+        <v>11</v>
+      </c>
+      <c r="D107" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>see</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>2</v>
+      </c>
+      <c r="C108" t="n">
+        <v>18</v>
+      </c>
+      <c r="D108" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>2</v>
+      </c>
+      <c r="C109" t="n">
+        <v>13</v>
+      </c>
+      <c r="D109" t="n">
+        <v>0.5925925925925926</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>3</v>
+      </c>
+      <c r="C110" t="n">
+        <v>28</v>
+      </c>
+      <c r="D110" t="n">
+        <v>1.488888888888889</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>trustpilot</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>3</v>
+      </c>
+      <c r="C111" t="n">
+        <v>18</v>
+      </c>
+      <c r="D111" t="n">
+        <v>1.063888888888889</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>from</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>2</v>
+      </c>
+      <c r="C112" t="n">
+        <v>13</v>
+      </c>
+      <c r="D112" t="n">
+        <v>0.5925925925925926</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>my</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>2</v>
+      </c>
+      <c r="C113" t="n">
+        <v>9</v>
+      </c>
+      <c r="D113" t="n">
+        <v>0.4592592592592592</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>2</v>
+      </c>
+      <c r="C114" t="n">
+        <v>10</v>
+      </c>
+      <c r="D114" t="n">
+        <v>0.5092592592592592</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>but</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>2</v>
+      </c>
+      <c r="C115" t="n">
+        <v>8</v>
+      </c>
+      <c r="D115" t="n">
+        <v>0.4537037037037037</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>platform</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>3</v>
+      </c>
+      <c r="C116" t="n">
+        <v>14</v>
+      </c>
+      <c r="D116" t="n">
+        <v>0.9662698412698413</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>credit</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>2</v>
+      </c>
+      <c r="C117" t="n">
+        <v>9</v>
+      </c>
+      <c r="D117" t="n">
+        <v>0.4351851851851852</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>2</v>
+      </c>
+      <c r="C118" t="n">
+        <v>17</v>
+      </c>
+      <c r="D118" t="n">
+        <v>0.6574074074074073</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>you re</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>2</v>
+      </c>
+      <c r="C119" t="n">
+        <v>9</v>
+      </c>
+      <c r="D119" t="n">
+        <v>0.8703703703703703</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>using</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>2</v>
+      </c>
+      <c r="C120" t="n">
+        <v>9</v>
+      </c>
+      <c r="D120" t="n">
+        <v>0.4351851851851852</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>2</v>
+      </c>
+      <c r="C121" t="n">
+        <v>6</v>
+      </c>
+      <c r="D121" t="n">
+        <v>0.3174603174603174</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>into</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>4</v>
+      </c>
+      <c r="C122" t="n">
+        <v>15</v>
+      </c>
+      <c r="D122" t="n">
+        <v>1.098412698412698</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>2</v>
+      </c>
+      <c r="C123" t="n">
+        <v>10</v>
+      </c>
+      <c r="D123" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>over</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>2</v>
+      </c>
+      <c r="C124" t="n">
+        <v>7</v>
+      </c>
+      <c r="D124" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>pricing</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>2</v>
+      </c>
+      <c r="C125" t="n">
+        <v>18</v>
+      </c>
+      <c r="D125" t="n">
+        <v>0.6388888888888888</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>ranking</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>2</v>
+      </c>
+      <c r="C126" t="n">
+        <v>11</v>
+      </c>
+      <c r="D126" t="n">
+        <v>0.4444444444444444</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>dataforseo com</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>2</v>
+      </c>
+      <c r="C127" t="n">
+        <v>6</v>
+      </c>
+      <c r="D127" t="n">
+        <v>0.6111111111111112</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>need</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>2</v>
+      </c>
+      <c r="C128" t="n">
+        <v>11</v>
+      </c>
+      <c r="D128" t="n">
+        <v>0.4444444444444444</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>automation</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>2</v>
+      </c>
+      <c r="C129" t="n">
+        <v>6</v>
+      </c>
+      <c r="D129" t="n">
+        <v>0.3174603174603174</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>3</v>
+      </c>
+      <c r="C130" t="n">
+        <v>10</v>
+      </c>
+      <c r="D130" t="n">
+        <v>0.6428571428571428</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>2</v>
+      </c>
+      <c r="C131" t="n">
+        <v>20</v>
+      </c>
+      <c r="D131" t="n">
+        <v>0.6944444444444444</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>across</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>2</v>
+      </c>
+      <c r="C132" t="n">
+        <v>11</v>
+      </c>
+      <c r="D132" t="n">
+        <v>0.4444444444444444</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>semrush</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>2</v>
+      </c>
+      <c r="C133" t="n">
+        <v>18</v>
+      </c>
+      <c r="D133" t="n">
+        <v>0.6388888888888888</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>than</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>2</v>
+      </c>
+      <c r="C134" t="n">
+        <v>18</v>
+      </c>
+      <c r="D134" t="n">
+        <v>0.6388888888888888</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>does</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>2</v>
+      </c>
+      <c r="C135" t="n">
+        <v>14</v>
+      </c>
+      <c r="D135" t="n">
+        <v>0.5277777777777778</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>while</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>2</v>
+      </c>
+      <c r="C136" t="n">
+        <v>7</v>
+      </c>
+      <c r="D136" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>logiciel</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>2</v>
+      </c>
+      <c r="C137" t="n">
+        <v>13</v>
+      </c>
+      <c r="D137" t="n">
+        <v>0.5061728395061729</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>référencement</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>2</v>
+      </c>
+      <c r="C138" t="n">
+        <v>10</v>
+      </c>
+      <c r="D138" t="n">
+        <v>1.111111111111111</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>intégrations</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>2</v>
+      </c>
+      <c r="C139" t="n">
+        <v>7</v>
+      </c>
+      <c r="D139" t="n">
+        <v>0.5308641975308642</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>2</v>
+      </c>
+      <c r="C140" t="n">
+        <v>10</v>
+      </c>
+      <c r="D140" t="n">
+        <v>0.3395061728395061</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>avis</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>2</v>
+      </c>
+      <c r="C141" t="n">
+        <v>14</v>
+      </c>
+      <c r="D141" t="n">
+        <v>0.4382716049382716</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>référencement gratuit</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>2</v>
+      </c>
+      <c r="C142" t="n">
+        <v>8</v>
+      </c>
+      <c r="D142" t="n">
+        <v>1.160493827160494</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>logiciel référencement</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>2</v>
+      </c>
+      <c r="C143" t="n">
+        <v>6</v>
+      </c>
+      <c r="D143" t="n">
+        <v>0.9629629629629629</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>logiciel référencement gratuit</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>2</v>
+      </c>
+      <c r="C144" t="n">
+        <v>6</v>
+      </c>
+      <c r="D144" t="n">
+        <v>1.203703703703703</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>utilisateur</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>2</v>
+      </c>
+      <c r="C145" t="n">
+        <v>8</v>
+      </c>
+      <c r="D145" t="n">
+        <v>0.2345679012345679</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>integration</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>2</v>
+      </c>
+      <c r="C146" t="n">
+        <v>26</v>
+      </c>
+      <c r="D146" t="n">
+        <v>0.7817460317460317</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>2</v>
+      </c>
+      <c r="C147" t="n">
+        <v>9</v>
+      </c>
+      <c r="D147" t="n">
+        <v>0.2738095238095238</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>2</v>
+      </c>
+      <c r="C148" t="n">
+        <v>8</v>
+      </c>
+      <c r="D148" t="n">
+        <v>0.242063492063492</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>no-code</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>2</v>
+      </c>
+      <c r="C149" t="n">
+        <v>8</v>
+      </c>
+      <c r="D149" t="n">
+        <v>0.4841269841269841</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>connect</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>2</v>
+      </c>
+      <c r="C150" t="n">
+        <v>9</v>
+      </c>
+      <c r="D150" t="n">
+        <v>0.2658730158730159</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>mcp</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>2</v>
+      </c>
+      <c r="C151" t="n">
+        <v>6</v>
+      </c>
+      <c r="D151" t="n">
+        <v>0.1785714285714286</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>sheets</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>2</v>
+      </c>
+      <c r="C152" t="n">
+        <v>8</v>
+      </c>
+      <c r="D152" t="n">
+        <v>0.2341269841269841</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>google</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>3</v>
+      </c>
+      <c r="C153" t="n">
+        <v>29</v>
+      </c>
+      <c r="D153" t="n">
+        <v>1.117857142857143</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>google sheets</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>2</v>
+      </c>
+      <c r="C154" t="n">
+        <v>8</v>
+      </c>
+      <c r="D154" t="n">
+        <v>0.4682539682539683</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>connect dataforseo to</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>2</v>
+      </c>
+      <c r="C155" t="n">
+        <v>4</v>
+      </c>
+      <c r="D155" t="n">
+        <v>0.3571428571428572</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>analysis</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>2</v>
+      </c>
+      <c r="C156" t="n">
+        <v>10</v>
+      </c>
+      <c r="D156" t="n">
+        <v>0.2611111111111111</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>alternatives</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>2</v>
+      </c>
+      <c r="C157" t="n">
+        <v>7</v>
+      </c>
+      <c r="D157" t="n">
+        <v>0.1851851851851852</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>2</v>
+      </c>
+      <c r="C158" t="n">
+        <v>9</v>
+      </c>
+      <c r="D158" t="n">
+        <v>0.2314814814814815</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>reviews api</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>2</v>
+      </c>
+      <c r="C159" t="n">
+        <v>6</v>
+      </c>
+      <c r="D159" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>google reviews api</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>2</v>
+      </c>
+      <c r="C160" t="n">
+        <v>5</v>
+      </c>
+      <c r="D160" t="n">
+        <v>0.3833333333333333</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Page position</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://nextgrowth.ai/dataforseo-review/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Is DataForSEO data accurate?</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>DataForSEO data is generally accurate, see how it compares to SerpApi in our DataForSEO vs SerpApi comparison for SERP results, keyword rankings, and Google Reviews. The platform pulls live data from search engines, improving freshness during algorithm updates. G2 reviews consistently rate accuracy highly (4+ stars). However, for backlink analysis specifically, Ahrefs’ larger index provides more comprehensive coverage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://nextgrowth.ai/dataforseo-review/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>How much does DataForSEO cost?</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>DataForSEO uses a pay-as-you-go pricing model with a $50 minimum deposit and no monthly fee. Standard queue SERP requests cost $0.0006 per request (DataForSEO Pricing, 2026). Agencies processing 5,000 requests/month typically spend ~$3/month. Costs scale directly with usage volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://nextgrowth.ai/dataforseo-review/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Is DataForSEO better than Ahrefs?</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>DataForSEO is better than Ahrefs for developers needing API access at a lower cost (often 70 ‐ 90% cheaper). Ahrefs offers a superior visual dashboard for non-technical users. The choice depends on whether your team can handle an API-first workflow via n8n or code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://nextgrowth.ai/dataforseo-review/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Does DataForSEO have a Google Reviews API?</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Yes, DataForSEO offers a dedicated Google Reviews API retrieving real-time reviews from Google My Business. It supports reputation management software and local SEO dashboards. Developers on G2 cite this as a unique strength. Access requires a standard account and credits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://nextgrowth.ai/dataforseo-review/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Is DataForSEO hard to use?</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>DataForSEO has a steeper learning curve than all-in-one tools because it lacks a built-in dashboard. Setup takes a few hours for developers, or under 30 minutes via n8n for non-coders. Reviewers note the initial effort is offset by long-term cost savings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>16</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://thatmarketingbuddy.com/software/dataforseo</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>What's the minimum cost to try DataForSEO?</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>$50 minimum payment. You can't test with smaller amounts, making this unsuitable for quick trials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://thatmarketingbuddy.com/software/dataforseo</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Do I need developers to use DataForSEO?</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Yes. This is an API platform that requires technical implementation, not a ready-to-use SEO tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>16</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://thatmarketingbuddy.com/software/dataforseo</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>How does pricing work exactly?</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Pay-per-request model where different API calls consume different amounts of credits. Costs vary significantly based on data complexity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>16</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://thatmarketingbuddy.com/software/dataforseo</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Can I build my own SEO tool with this data?</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Absolutely. That's the main use case. DataForSEO provides the data infrastructure for custom SEO applications.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>16</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://thatmarketingbuddy.com/software/dataforseo</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>How fresh is the data compared to other SEO tools?</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Very fresh. Keywords update within 30 days, backlinks are crawled continuously, and SERP data reflects real-time results.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>16</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://thatmarketingbuddy.com/software/dataforseo</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Is there a free trial or free tier?</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>No traditional free trial, but you can register and explore the documentation. All data access requires the $50 minimum payment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>16</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://thatmarketingbuddy.com/software/dataforseo</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>What makes this different from Ahrefs or Semrush APIs?</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>More comprehensive API coverage (11 different categories), fresher data updates, and designed API-first rather than as platform extensions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>16</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://thatmarketingbuddy.com/software/dataforseo</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Can small businesses use this effectively?</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Generally not. The technical requirements and minimum costs make it better suited for software companies, agencies, or enterprises with development resources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>16</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://thatmarketingbuddy.com/software/dataforseo</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Does DataForSEO have AI features?</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MCP server available, making DataForSEO directly accessible from Claude Desktop, Cursor, and other AI coding tools. REST API adds a second automation path for custom AI workflows.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>